<commit_message>
updated rhynie metaweb builder pipeline
converted adj_matrix_builder_rhynie to metaweb_builder_rhynie.R

the new file takes the updated Excel workbook and generates a guilds, links, and matrix csv, as well as a lumped version
</commit_message>
<xml_diff>
--- a/data/rhynie/RhynieGuildStructure.xlsx
+++ b/data/rhynie/RhynieGuildStructure.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tannerfrank/Dropbox/Work/Devonian terr ecosystems/EcolNetworks/RhynieWebRepo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tannerfrank/Dropbox/Work/Devonian terr ecosystems/EcolNetworks/RhynieWebRepo/data/rhynie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334E4D07-7CAA-8B45-AC52-8FA729F4BB0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04812DE6-19A8-1B4A-BB07-6A41C4F78623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="16000" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guilds" sheetId="1" r:id="rId1"/>
     <sheet name="Guild composition" sheetId="2" r:id="rId2"/>
+    <sheet name="Lumped priority" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="265">
   <si>
     <t>guild_no</t>
   </si>
@@ -35,15 +36,6 @@
     <t>G</t>
   </si>
   <si>
-    <t>priority resource guild(s)</t>
-  </si>
-  <si>
-    <t>general resource guilds(s)</t>
-  </si>
-  <si>
-    <t>resource_guilds_original</t>
-  </si>
-  <si>
     <t>terr</t>
   </si>
   <si>
@@ -771,6 +763,60 @@
   </si>
   <si>
     <t>22,23,25,26</t>
+  </si>
+  <si>
+    <t>lumped_id</t>
+  </si>
+  <si>
+    <t>lumped_G</t>
+  </si>
+  <si>
+    <t>lumped_name</t>
+  </si>
+  <si>
+    <t>land plants</t>
+  </si>
+  <si>
+    <t>terrestrial microbes</t>
+  </si>
+  <si>
+    <t>terrestrial fungi</t>
+  </si>
+  <si>
+    <t>aquatic heterotrophic microbes</t>
+  </si>
+  <si>
+    <t>aquatic algae</t>
+  </si>
+  <si>
+    <t>aquatic fungi</t>
+  </si>
+  <si>
+    <t>consumer_lumped_id</t>
+  </si>
+  <si>
+    <t>resource_lumped_id</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>priority_resources</t>
+  </si>
+  <si>
+    <t>general_resources</t>
+  </si>
+  <si>
+    <t>microbes play a major role as decomposers</t>
+  </si>
+  <si>
+    <t>saprotrophy is the canonical feeding mode of fungi in food webs</t>
+  </si>
+  <si>
+    <t>resources_old</t>
+  </si>
+  <si>
+    <t>priority</t>
   </si>
 </sst>
 </file>
@@ -924,7 +970,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -974,7 +1020,6 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2105,21 +2150,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="5.83203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="42.1640625" style="1" customWidth="1"/>
-    <col min="8" max="10" width="10.83203125" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="1"/>
+    <col min="4" max="5" width="5.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="1" customWidth="1"/>
+    <col min="10" max="11" width="10.83203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2133,1243 +2181,1710 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="L1" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
+      <c r="E2" s="3">
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="3">
-        <v>1</v>
-      </c>
-      <c r="I2" s="3">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="3">
+        <v>1</v>
+      </c>
+      <c r="K2" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="3">
-        <v>1</v>
-      </c>
-      <c r="I3" s="3">
+      <c r="E3" s="3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" s="3">
-        <v>1</v>
-      </c>
-      <c r="I4" s="3">
+      <c r="E4" s="3">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="3">
+        <v>1</v>
+      </c>
+      <c r="K4" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="3">
-        <v>1</v>
-      </c>
-      <c r="I5" s="3">
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G5" s="3">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="3">
+        <v>1</v>
+      </c>
+      <c r="K5" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" s="3">
-        <v>1</v>
-      </c>
-      <c r="I6" s="3">
+      <c r="E6" s="3">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G6" s="3">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="3">
+        <v>1</v>
+      </c>
+      <c r="K6" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="3">
-        <v>1</v>
-      </c>
-      <c r="I7" s="3">
+      <c r="E7" s="3">
+        <v>2</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G7" s="3">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="3">
+        <v>1</v>
+      </c>
+      <c r="K7" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3">
         <v>2</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="3">
-        <v>1</v>
-      </c>
-      <c r="I8" s="3">
+      <c r="E8" s="3">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G8" s="3">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" s="3">
+        <v>1</v>
+      </c>
+      <c r="K8" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L8" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="3">
         <v>1</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="3">
-        <v>1</v>
-      </c>
-      <c r="I9" s="3">
+      <c r="E9" s="3">
+        <v>2</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1</v>
+      </c>
+      <c r="K9" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="3">
         <v>1</v>
       </c>
       <c r="E10" s="3">
-        <v>1</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>22</v>
+        <v>3</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1</v>
       </c>
       <c r="H10" s="3">
         <v>1</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="3">
+        <v>1</v>
+      </c>
+      <c r="K10" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="3">
         <v>1</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="3">
-        <v>1</v>
-      </c>
-      <c r="I11" s="3">
+      <c r="E11" s="3">
+        <v>3</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G11" s="3">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="3">
+        <v>1</v>
+      </c>
+      <c r="K11" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D12" s="3">
         <v>14</v>
       </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="3">
-        <v>1</v>
+      <c r="E12" s="3">
+        <v>4</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>252</v>
       </c>
       <c r="G12" s="3">
         <v>1</v>
       </c>
-      <c r="H12" s="3">
-        <v>1</v>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="I12" s="3">
+        <v>1</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1</v>
+      </c>
+      <c r="K12" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="3">
         <v>3</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3">
-        <v>1</v>
-      </c>
-      <c r="I13" s="3">
+      <c r="E13" s="3">
+        <v>4</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="3">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="3">
+        <v>1</v>
+      </c>
+      <c r="K13" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="3">
         <v>2</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="3">
-        <v>1</v>
-      </c>
-      <c r="I14" s="3">
+      <c r="E14" s="3">
+        <v>4</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="3">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" s="3">
+        <v>1</v>
+      </c>
+      <c r="K14" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="3">
         <v>3</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="3">
-        <v>1</v>
-      </c>
-      <c r="I15" s="3">
+      <c r="E15" s="3">
+        <v>4</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="3">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J15" s="3">
+        <v>1</v>
+      </c>
+      <c r="K15" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="3">
         <v>3</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="3">
-        <v>1</v>
-      </c>
-      <c r="I16" s="3">
+      <c r="E16" s="3">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G16" s="3">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J16" s="3">
+        <v>1</v>
+      </c>
+      <c r="K16" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3">
+        <v>4</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G17" s="3">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J17" s="3">
+        <v>1</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="3">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="3">
-        <v>1</v>
-      </c>
-      <c r="I17" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="3">
         <v>1</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="3">
-        <v>1</v>
-      </c>
-      <c r="I18" s="3">
+      <c r="E18" s="3">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G18" s="3">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J18" s="3">
+        <v>1</v>
+      </c>
+      <c r="K18" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="3">
         <v>3</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G19" s="2"/>
-      <c r="H19" s="3">
-        <v>1</v>
-      </c>
-      <c r="I19" s="3">
+      <c r="E19" s="3">
+        <v>4</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G19" s="3">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J19" s="3">
+        <v>1</v>
+      </c>
+      <c r="K19" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="3">
         <v>1</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="3">
-        <v>1</v>
-      </c>
-      <c r="I20" s="3">
+      <c r="E20" s="3">
+        <v>4</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G20" s="3">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J20" s="3">
+        <v>1</v>
+      </c>
+      <c r="K20" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D21" s="3">
         <v>2</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H21" s="3">
-        <v>1</v>
-      </c>
-      <c r="I21" s="3">
+      <c r="E21" s="3">
+        <v>4</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G21" s="3">
+        <v>1</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="3">
+        <v>1</v>
+      </c>
+      <c r="K21" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L21" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D22" s="3">
         <v>7</v>
       </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H22" s="3">
-        <v>1</v>
-      </c>
-      <c r="I22" s="3">
+      <c r="E22" s="3">
+        <v>4</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G22" s="3">
+        <v>1</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J22" s="3">
+        <v>1</v>
+      </c>
+      <c r="K22" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L22" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="3">
         <v>1</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>29</v>
+      <c r="E23" s="3">
+        <v>5</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="3">
-        <v>1</v>
-      </c>
-      <c r="I23" s="3">
+        <v>54</v>
+      </c>
+      <c r="G23" s="3">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J23" s="3">
+        <v>1</v>
+      </c>
+      <c r="K23" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="3">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3">
+        <v>6</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J24" s="3">
+        <v>1</v>
+      </c>
+      <c r="K24" s="3">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="3">
-        <v>1</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H24" s="3">
-        <v>1</v>
-      </c>
-      <c r="I24" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D25" s="3">
         <v>2</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>65</v>
+      <c r="E25" s="3">
+        <v>7</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H25" s="3">
-        <v>1</v>
-      </c>
-      <c r="I25" s="3">
+        <v>60</v>
+      </c>
+      <c r="G25" s="3">
+        <v>2</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J25" s="3">
+        <v>1</v>
+      </c>
+      <c r="K25" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L25" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D26" s="3">
         <v>2</v>
       </c>
-      <c r="E26" s="2"/>
+      <c r="E26" s="3">
+        <v>8</v>
+      </c>
       <c r="F26" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="H26" s="3">
-        <v>1</v>
-      </c>
-      <c r="I26" s="3">
+        <v>65</v>
+      </c>
+      <c r="G26" s="3">
+        <v>2</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="J26" s="3">
+        <v>1</v>
+      </c>
+      <c r="K26" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L26" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D27" s="3">
         <v>3</v>
       </c>
-      <c r="E27" s="2"/>
+      <c r="E27" s="3">
+        <v>9</v>
+      </c>
       <c r="F27" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H27" s="3">
-        <v>1</v>
-      </c>
-      <c r="I27" s="3">
+        <v>69</v>
+      </c>
+      <c r="G27" s="3">
+        <v>3</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="J27" s="3">
+        <v>1</v>
+      </c>
+      <c r="K27" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L27" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D28" s="3">
         <v>5</v>
       </c>
-      <c r="E28" s="2"/>
+      <c r="E28" s="3">
+        <v>10</v>
+      </c>
       <c r="F28" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H28" s="3">
-        <v>1</v>
-      </c>
-      <c r="I28" s="3">
+        <v>72</v>
+      </c>
+      <c r="G28" s="3">
+        <v>5</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J28" s="3">
+        <v>1</v>
+      </c>
+      <c r="K28" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L28" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D29" s="3">
         <v>1</v>
       </c>
-      <c r="E29" s="2"/>
+      <c r="E29" s="3">
+        <v>11</v>
+      </c>
       <c r="F29" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H29" s="3">
+        <v>76</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J29" s="3">
         <v>0</v>
       </c>
-      <c r="I29" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K29" s="3">
+        <v>1</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="3">
         <v>1</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="H30" s="3">
+      <c r="E30" s="3">
+        <v>12</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="G30" s="3">
+        <v>1</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J30" s="3">
         <v>0</v>
       </c>
-      <c r="I30" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K30" s="3">
+        <v>1</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="3">
         <v>1</v>
       </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="2" t="s">
+      <c r="E31" s="3">
         <v>12</v>
       </c>
-      <c r="G31" s="5"/>
-      <c r="H31" s="3">
+      <c r="F31" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="G31" s="3">
+        <v>1</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J31" s="3">
         <v>0</v>
       </c>
-      <c r="I31" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K31" s="3">
+        <v>1</v>
+      </c>
+      <c r="L31" s="5"/>
+    </row>
+    <row r="32" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="3">
         <v>1</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="3">
+      <c r="E32" s="3">
+        <v>12</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="G32" s="3">
+        <v>1</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="J32" s="3">
         <v>0</v>
       </c>
-      <c r="I32" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K32" s="3">
+        <v>1</v>
+      </c>
+      <c r="L32" s="5"/>
+    </row>
+    <row r="33" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="3">
         <v>1</v>
       </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="5"/>
-      <c r="H33" s="3">
+      <c r="E33" s="3">
+        <v>13</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G33" s="3">
+        <v>1</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J33" s="3">
         <v>0</v>
       </c>
-      <c r="I33" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K33" s="3">
+        <v>1</v>
+      </c>
+      <c r="L33" s="5"/>
+    </row>
+    <row r="34" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D34" s="3">
         <v>5</v>
       </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="5"/>
-      <c r="H34" s="3">
+      <c r="E34" s="3">
+        <v>13</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G34" s="3">
+        <v>1</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J34" s="3">
         <v>0</v>
       </c>
-      <c r="I34" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K34" s="3">
+        <v>1</v>
+      </c>
+      <c r="L34" s="5"/>
+    </row>
+    <row r="35" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
       </c>
-      <c r="E35" s="5"/>
-      <c r="F35" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G35" s="5"/>
-      <c r="H35" s="3">
+      <c r="E35" s="3">
+        <v>13</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G35" s="3">
+        <v>1</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J35" s="3">
         <v>0</v>
       </c>
-      <c r="I35" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K35" s="3">
+        <v>1</v>
+      </c>
+      <c r="L35" s="5"/>
+    </row>
+    <row r="36" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D36" s="3">
         <v>5</v>
       </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="5"/>
-      <c r="H36" s="3">
+      <c r="E36" s="3">
+        <v>13</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G36" s="3">
+        <v>1</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J36" s="3">
         <v>0</v>
       </c>
-      <c r="I36" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K36" s="3">
+        <v>1</v>
+      </c>
+      <c r="L36" s="5"/>
+    </row>
+    <row r="37" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D37" s="3">
         <v>4</v>
       </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="5"/>
-      <c r="H37" s="3">
+      <c r="E37" s="3">
+        <v>13</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G37" s="3">
+        <v>1</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J37" s="3">
         <v>0</v>
       </c>
-      <c r="I37" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K37" s="3">
+        <v>1</v>
+      </c>
+      <c r="L37" s="5"/>
+    </row>
+    <row r="38" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D38" s="3">
         <v>1</v>
       </c>
-      <c r="E38" s="5"/>
-      <c r="F38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G38" s="5"/>
-      <c r="H38" s="3">
+      <c r="E38" s="3">
+        <v>14</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G38" s="3">
+        <v>1</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J38" s="3">
         <v>0</v>
       </c>
-      <c r="I38" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K38" s="3">
+        <v>1</v>
+      </c>
+      <c r="L38" s="5"/>
+    </row>
+    <row r="39" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D39" s="3">
         <v>3</v>
       </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G39" s="5"/>
-      <c r="H39" s="3">
-        <v>1</v>
-      </c>
-      <c r="I39" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E39" s="3">
+        <v>13</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G39" s="3">
+        <v>1</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J39" s="3">
+        <v>1</v>
+      </c>
+      <c r="K39" s="3">
+        <v>1</v>
+      </c>
+      <c r="L39" s="5"/>
+    </row>
+    <row r="40" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D40" s="3">
         <v>5</v>
       </c>
-      <c r="E40" s="5"/>
-      <c r="F40" s="3">
+      <c r="E40" s="3">
+        <v>15</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="G40" s="3">
+        <v>1</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I40" s="3">
         <v>28</v>
       </c>
-      <c r="G40" s="3">
+      <c r="J40" s="3">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3">
+        <v>1</v>
+      </c>
+      <c r="L40" s="3">
         <v>13</v>
       </c>
-      <c r="H40" s="3">
-        <v>0</v>
-      </c>
-      <c r="I40" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D41" s="3">
+        <v>1</v>
+      </c>
+      <c r="E41" s="3">
+        <v>15</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="G41" s="3">
+        <v>1</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3">
+        <v>1</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D41" s="3">
-        <v>1</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H41" s="3">
-        <v>0</v>
-      </c>
-      <c r="I41" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D42" s="3">
         <v>1</v>
       </c>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="H42" s="3">
+      <c r="E42" s="3">
+        <v>15</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="G42" s="3">
+        <v>1</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J42" s="3">
         <v>0</v>
       </c>
-      <c r="I42" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K42" s="3">
+        <v>1</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D43" s="3">
+        <v>1</v>
+      </c>
+      <c r="E43" s="3">
+        <v>16</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G43" s="3">
+        <v>1</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="J43" s="3">
+        <v>0</v>
+      </c>
+      <c r="K43" s="3">
+        <v>1</v>
+      </c>
+      <c r="L43" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D43" s="3">
-        <v>1</v>
-      </c>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="H43" s="3">
-        <v>1</v>
-      </c>
-      <c r="I43" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D44" s="3">
         <v>2</v>
       </c>
-      <c r="E44" s="2"/>
+      <c r="E44" s="3">
+        <v>17</v>
+      </c>
       <c r="F44" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H44" s="3">
+        <v>108</v>
+      </c>
+      <c r="G44" s="3">
+        <v>2</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J44" s="3">
         <v>0</v>
       </c>
-      <c r="I44" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K44" s="3">
+        <v>1</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45" s="3">
+        <v>1</v>
+      </c>
+      <c r="E45" s="3">
+        <v>18</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G45" s="3">
+        <v>1</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J45" s="3">
+        <v>0</v>
+      </c>
+      <c r="K45" s="3">
+        <v>1</v>
+      </c>
+      <c r="L45" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D45" s="3">
-        <v>1</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="H45" s="3">
-        <v>0</v>
-      </c>
-      <c r="I45" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D46" s="3">
         <v>2</v>
       </c>
-      <c r="E46" s="2"/>
+      <c r="E46" s="3">
+        <v>19</v>
+      </c>
       <c r="F46" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H46" s="3">
+        <v>116</v>
+      </c>
+      <c r="G46" s="3">
+        <v>2</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="J46" s="3">
         <v>0</v>
       </c>
-      <c r="I46" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K46" s="3">
+        <v>1</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D47" s="3">
+        <v>1</v>
+      </c>
+      <c r="E47" s="3">
+        <v>20</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G47" s="3">
+        <v>1</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="3">
+        <v>1</v>
+      </c>
+      <c r="L47" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D47" s="3">
-        <v>1</v>
-      </c>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H47" s="3">
-        <v>0</v>
-      </c>
-      <c r="I47" s="3">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3395,16 +3910,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="E1" s="5"/>
     </row>
@@ -3413,7 +3928,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2" s="7">
         <v>1</v>
@@ -3425,7 +3940,7 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="5"/>
@@ -3435,7 +3950,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -3447,7 +3962,7 @@
       <c r="A5" s="9"/>
       <c r="B5" s="4"/>
       <c r="C5" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="5"/>
@@ -3457,7 +3972,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C6" s="7">
         <v>1</v>
@@ -3469,7 +3984,7 @@
       <c r="A7" s="9"/>
       <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="5"/>
@@ -3479,7 +3994,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
@@ -3491,7 +4006,7 @@
       <c r="A9" s="9"/>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="5"/>
@@ -3501,7 +4016,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -3513,7 +4028,7 @@
       <c r="A11" s="9"/>
       <c r="B11" s="4"/>
       <c r="C11" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="5"/>
@@ -3523,7 +4038,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
@@ -3535,7 +4050,7 @@
       <c r="A13" s="9"/>
       <c r="B13" s="6"/>
       <c r="C13" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="5"/>
@@ -3545,7 +4060,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C14" s="7">
         <v>2</v>
@@ -3557,7 +4072,7 @@
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="10" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="5"/>
@@ -3566,7 +4081,7 @@
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="10" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="5"/>
@@ -3583,10 +4098,10 @@
         <v>8</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="5"/>
@@ -3595,7 +4110,7 @@
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="10" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="5"/>
@@ -3605,7 +4120,7 @@
         <v>9</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C20" s="7">
         <v>1</v>
@@ -3617,7 +4132,7 @@
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="10" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="5"/>
@@ -3627,7 +4142,7 @@
         <v>10</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C22" s="13">
         <v>1</v>
@@ -3639,10 +4154,10 @@
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="10" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E23" s="5"/>
     </row>
@@ -3651,7 +4166,7 @@
         <v>11</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C24" s="7">
         <v>14</v>
@@ -3663,7 +4178,7 @@
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="5"/>
@@ -3672,10 +4187,10 @@
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E26" s="5"/>
     </row>
@@ -3683,10 +4198,10 @@
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="10" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E27" s="5"/>
     </row>
@@ -3694,10 +4209,10 @@
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E28" s="5"/>
     </row>
@@ -3705,10 +4220,10 @@
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E29" s="5"/>
     </row>
@@ -3716,10 +4231,10 @@
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E30" s="5"/>
     </row>
@@ -3727,7 +4242,7 @@
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="10" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="5"/>
@@ -3736,7 +4251,7 @@
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="10" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="5"/>
@@ -3745,7 +4260,7 @@
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="10" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="5"/>
@@ -3754,16 +4269,16 @@
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="D34" s="27"/>
+        <v>150</v>
+      </c>
+      <c r="D34" s="5"/>
       <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="5"/>
@@ -3772,7 +4287,7 @@
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="5"/>
@@ -3781,10 +4296,10 @@
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E37" s="5"/>
     </row>
@@ -3792,10 +4307,10 @@
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="10" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E38" s="5"/>
     </row>
@@ -3804,7 +4319,7 @@
         <v>12</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C39" s="7">
         <v>3</v>
@@ -3816,7 +4331,7 @@
       <c r="A40" s="9"/>
       <c r="B40" s="6"/>
       <c r="C40" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="5"/>
@@ -3825,7 +4340,7 @@
       <c r="A41" s="9"/>
       <c r="B41" s="6"/>
       <c r="C41" s="10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="5"/>
@@ -3834,7 +4349,7 @@
       <c r="A42" s="9"/>
       <c r="B42" s="6"/>
       <c r="C42" s="10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="5"/>
@@ -3844,7 +4359,7 @@
         <v>13</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C43" s="7">
         <v>2</v>
@@ -3856,7 +4371,7 @@
       <c r="A44" s="9"/>
       <c r="B44" s="6"/>
       <c r="C44" s="15" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="5"/>
@@ -3865,7 +4380,7 @@
       <c r="A45" s="9"/>
       <c r="B45" s="6"/>
       <c r="C45" s="10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="5"/>
@@ -3875,7 +4390,7 @@
         <v>14</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C46" s="7">
         <v>3</v>
@@ -3887,7 +4402,7 @@
       <c r="A47" s="9"/>
       <c r="B47" s="6"/>
       <c r="C47" s="15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="5"/>
@@ -3896,7 +4411,7 @@
       <c r="A48" s="9"/>
       <c r="B48" s="6"/>
       <c r="C48" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="5"/>
@@ -3905,7 +4420,7 @@
       <c r="A49" s="9"/>
       <c r="B49" s="6"/>
       <c r="C49" s="10" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="5"/>
@@ -3915,7 +4430,7 @@
         <v>15</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C50" s="7">
         <v>3</v>
@@ -3927,7 +4442,7 @@
       <c r="A51" s="9"/>
       <c r="B51" s="6"/>
       <c r="C51" s="10" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="5"/>
@@ -3936,7 +4451,7 @@
       <c r="A52" s="9"/>
       <c r="B52" s="6"/>
       <c r="C52" s="10" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="5"/>
@@ -3945,7 +4460,7 @@
       <c r="A53" s="9"/>
       <c r="B53" s="6"/>
       <c r="C53" s="10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="5"/>
@@ -3955,7 +4470,7 @@
         <v>16</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C54" s="7">
         <v>1</v>
@@ -3967,10 +4482,10 @@
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="10" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E55" s="5"/>
     </row>
@@ -3979,7 +4494,7 @@
         <v>17</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C56" s="7">
         <v>1</v>
@@ -3991,7 +4506,7 @@
       <c r="A57" s="9"/>
       <c r="B57" s="6"/>
       <c r="C57" s="10" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D57" s="8"/>
       <c r="E57" s="5"/>
@@ -4001,7 +4516,7 @@
         <v>18</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C58" s="7">
         <v>3</v>
@@ -4013,10 +4528,10 @@
       <c r="A59" s="9"/>
       <c r="B59" s="6"/>
       <c r="C59" s="10" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E59" s="5"/>
     </row>
@@ -4024,7 +4539,7 @@
       <c r="A60" s="9"/>
       <c r="B60" s="6"/>
       <c r="C60" s="10" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D60" s="8"/>
       <c r="E60" s="5"/>
@@ -4033,7 +4548,7 @@
       <c r="A61" s="9"/>
       <c r="B61" s="6"/>
       <c r="C61" s="10" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D61" s="8"/>
       <c r="E61" s="5"/>
@@ -4043,7 +4558,7 @@
         <v>19</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C62" s="7">
         <v>1</v>
@@ -4055,10 +4570,10 @@
       <c r="A63" s="9"/>
       <c r="B63" s="6"/>
       <c r="C63" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E63" s="5"/>
     </row>
@@ -4067,7 +4582,7 @@
         <v>20</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C64" s="7">
         <v>2</v>
@@ -4079,7 +4594,7 @@
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="10" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
@@ -4088,10 +4603,10 @@
       <c r="A66" s="8"/>
       <c r="B66" s="8"/>
       <c r="C66" s="10" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E66" s="5"/>
     </row>
@@ -4100,7 +4615,7 @@
         <v>21</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C67" s="7">
         <v>7</v>
@@ -4112,10 +4627,10 @@
       <c r="A68" s="8"/>
       <c r="B68" s="8"/>
       <c r="C68" s="10" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E68" s="5"/>
     </row>
@@ -4123,10 +4638,10 @@
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E69" s="5"/>
     </row>
@@ -4134,10 +4649,10 @@
       <c r="A70" s="8"/>
       <c r="B70" s="8"/>
       <c r="C70" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E70" s="5"/>
     </row>
@@ -4145,10 +4660,10 @@
       <c r="A71" s="8"/>
       <c r="B71" s="8"/>
       <c r="C71" s="10" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E71" s="5"/>
     </row>
@@ -4156,10 +4671,10 @@
       <c r="A72" s="8"/>
       <c r="B72" s="8"/>
       <c r="C72" s="10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E72" s="5"/>
     </row>
@@ -4167,10 +4682,10 @@
       <c r="A73" s="8"/>
       <c r="B73" s="8"/>
       <c r="C73" s="10" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E73" s="5"/>
     </row>
@@ -4178,10 +4693,10 @@
       <c r="A74" s="8"/>
       <c r="B74" s="8"/>
       <c r="C74" s="10" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E74" s="5"/>
     </row>
@@ -4190,7 +4705,7 @@
         <v>22</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C75" s="7">
         <v>1</v>
@@ -4202,7 +4717,7 @@
       <c r="A76" s="9"/>
       <c r="B76" s="6"/>
       <c r="C76" s="15" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D76" s="8"/>
       <c r="E76" s="5"/>
@@ -4212,7 +4727,7 @@
         <v>23</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C77" s="7">
         <v>1</v>
@@ -4224,7 +4739,7 @@
       <c r="A78" s="8"/>
       <c r="B78" s="8"/>
       <c r="C78" s="6" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D78" s="8"/>
       <c r="E78" s="5"/>
@@ -4234,7 +4749,7 @@
         <v>24</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C79" s="7">
         <v>2</v>
@@ -4246,10 +4761,10 @@
       <c r="A80" s="8"/>
       <c r="B80" s="8"/>
       <c r="C80" s="6" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E80" s="5"/>
     </row>
@@ -4257,7 +4772,7 @@
       <c r="A81" s="8"/>
       <c r="B81" s="8"/>
       <c r="C81" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D81" s="8"/>
       <c r="E81" s="5"/>
@@ -4267,7 +4782,7 @@
         <v>25</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C82" s="7">
         <v>2</v>
@@ -4279,10 +4794,10 @@
       <c r="A83" s="8"/>
       <c r="B83" s="8"/>
       <c r="C83" s="6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E83" s="5"/>
     </row>
@@ -4290,10 +4805,10 @@
       <c r="A84" s="8"/>
       <c r="B84" s="8"/>
       <c r="C84" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E84" s="5"/>
     </row>
@@ -4302,7 +4817,7 @@
         <v>26</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C85" s="7">
         <v>3</v>
@@ -4314,7 +4829,7 @@
       <c r="A86" s="8"/>
       <c r="B86" s="8"/>
       <c r="C86" s="6" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D86" s="8"/>
       <c r="E86" s="5"/>
@@ -4323,7 +4838,7 @@
       <c r="A87" s="8"/>
       <c r="B87" s="8"/>
       <c r="C87" s="6" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D87" s="8"/>
       <c r="E87" s="5"/>
@@ -4332,7 +4847,7 @@
       <c r="A88" s="8"/>
       <c r="B88" s="8"/>
       <c r="C88" s="6" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D88" s="8"/>
       <c r="E88" s="5"/>
@@ -4342,7 +4857,7 @@
         <v>27</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C89" s="7">
         <v>5</v>
@@ -4354,7 +4869,7 @@
       <c r="A90" s="8"/>
       <c r="B90" s="8"/>
       <c r="C90" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D90" s="8"/>
       <c r="E90" s="5"/>
@@ -4363,7 +4878,7 @@
       <c r="A91" s="8"/>
       <c r="B91" s="8"/>
       <c r="C91" s="6" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D91" s="8"/>
       <c r="E91" s="5"/>
@@ -4372,7 +4887,7 @@
       <c r="A92" s="8"/>
       <c r="B92" s="8"/>
       <c r="C92" s="6" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D92" s="8"/>
       <c r="E92" s="5"/>
@@ -4381,7 +4896,7 @@
       <c r="A93" s="8"/>
       <c r="B93" s="8"/>
       <c r="C93" s="6" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D93" s="8"/>
       <c r="E93" s="5"/>
@@ -4390,7 +4905,7 @@
       <c r="A94" s="8"/>
       <c r="B94" s="8"/>
       <c r="C94" s="6" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D94" s="8"/>
       <c r="E94" s="5"/>
@@ -4400,7 +4915,7 @@
         <v>28</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C95" s="7">
         <v>1</v>
@@ -4412,7 +4927,7 @@
       <c r="A96" s="8"/>
       <c r="B96" s="8"/>
       <c r="C96" s="6" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D96" s="8"/>
       <c r="E96" s="5"/>
@@ -4422,7 +4937,7 @@
         <v>29</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C97" s="7">
         <v>1</v>
@@ -4434,7 +4949,7 @@
       <c r="A98" s="8"/>
       <c r="B98" s="8"/>
       <c r="C98" s="6" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D98" s="8"/>
       <c r="E98" s="5"/>
@@ -4444,7 +4959,7 @@
         <v>30</v>
       </c>
       <c r="B99" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C99" s="7">
         <v>1</v>
@@ -4456,7 +4971,7 @@
       <c r="A100" s="8"/>
       <c r="B100" s="8"/>
       <c r="C100" s="6" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D100" s="8"/>
       <c r="E100" s="5"/>
@@ -4466,7 +4981,7 @@
         <v>31</v>
       </c>
       <c r="B101" s="12" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C101" s="3">
         <v>1</v>
@@ -4478,7 +4993,7 @@
       <c r="A102" s="8"/>
       <c r="B102" s="8"/>
       <c r="C102" s="10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D102" s="8"/>
       <c r="E102" s="5"/>
@@ -4488,7 +5003,7 @@
         <v>32</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C103" s="3">
         <v>1</v>
@@ -4500,7 +5015,7 @@
       <c r="A104" s="9"/>
       <c r="B104" s="6"/>
       <c r="C104" s="15" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D104" s="8"/>
       <c r="E104" s="5"/>
@@ -4510,7 +5025,7 @@
         <v>33</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C105" s="7">
         <v>5</v>
@@ -4522,7 +5037,7 @@
       <c r="A106" s="8"/>
       <c r="B106" s="8"/>
       <c r="C106" s="10" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D106" s="8"/>
       <c r="E106" s="5"/>
@@ -4531,7 +5046,7 @@
       <c r="A107" s="8"/>
       <c r="B107" s="8"/>
       <c r="C107" s="10" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D107" s="8"/>
       <c r="E107" s="5"/>
@@ -4540,7 +5055,7 @@
       <c r="A108" s="8"/>
       <c r="B108" s="8"/>
       <c r="C108" s="10" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="5"/>
@@ -4549,7 +5064,7 @@
       <c r="A109" s="8"/>
       <c r="B109" s="8"/>
       <c r="C109" s="10" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D109" s="8"/>
       <c r="E109" s="5"/>
@@ -4558,7 +5073,7 @@
       <c r="A110" s="8"/>
       <c r="B110" s="8"/>
       <c r="C110" s="10" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D110" s="8"/>
       <c r="E110" s="5"/>
@@ -4568,7 +5083,7 @@
         <v>34</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C111" s="7">
         <v>1</v>
@@ -4580,7 +5095,7 @@
       <c r="A112" s="8"/>
       <c r="B112" s="8"/>
       <c r="C112" s="10" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D112" s="8"/>
       <c r="E112" s="5"/>
@@ -4590,7 +5105,7 @@
         <v>35</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C113" s="7">
         <v>5</v>
@@ -4602,10 +5117,10 @@
       <c r="A114" s="8"/>
       <c r="B114" s="8"/>
       <c r="C114" s="10" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E114" s="5"/>
     </row>
@@ -4613,10 +5128,10 @@
       <c r="A115" s="8"/>
       <c r="B115" s="8"/>
       <c r="C115" s="10" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E115" s="5"/>
     </row>
@@ -4624,7 +5139,7 @@
       <c r="A116" s="8"/>
       <c r="B116" s="8"/>
       <c r="C116" s="10" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D116" s="8"/>
       <c r="E116" s="5"/>
@@ -4633,10 +5148,10 @@
       <c r="A117" s="8"/>
       <c r="B117" s="8"/>
       <c r="C117" s="10" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E117" s="5"/>
     </row>
@@ -4644,10 +5159,10 @@
       <c r="A118" s="8"/>
       <c r="B118" s="8"/>
       <c r="C118" s="10" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E118" s="5"/>
     </row>
@@ -4656,7 +5171,7 @@
         <v>36</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C119" s="7">
         <v>4</v>
@@ -4668,7 +5183,7 @@
       <c r="A120" s="8"/>
       <c r="B120" s="8"/>
       <c r="C120" s="10" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D120" s="8"/>
       <c r="E120" s="5"/>
@@ -4677,7 +5192,7 @@
       <c r="A121" s="8"/>
       <c r="B121" s="8"/>
       <c r="C121" s="10" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D121" s="8"/>
       <c r="E121" s="5"/>
@@ -4686,7 +5201,7 @@
       <c r="A122" s="8"/>
       <c r="B122" s="8"/>
       <c r="C122" s="10" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D122" s="8"/>
       <c r="E122" s="5"/>
@@ -4695,7 +5210,7 @@
       <c r="A123" s="8"/>
       <c r="B123" s="8"/>
       <c r="C123" s="10" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D123" s="8"/>
       <c r="E123" s="5"/>
@@ -4705,7 +5220,7 @@
         <v>37</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C124" s="7">
         <v>1</v>
@@ -4717,7 +5232,7 @@
       <c r="A125" s="8"/>
       <c r="B125" s="8"/>
       <c r="C125" s="10" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D125" s="8"/>
       <c r="E125" s="5"/>
@@ -4727,7 +5242,7 @@
         <v>38</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C126" s="16">
         <v>3</v>
@@ -4739,7 +5254,7 @@
       <c r="A127" s="8"/>
       <c r="B127" s="8"/>
       <c r="C127" s="10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D127" s="8"/>
       <c r="E127" s="5"/>
@@ -4748,7 +5263,7 @@
       <c r="A128" s="8"/>
       <c r="B128" s="8"/>
       <c r="C128" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D128" s="8"/>
       <c r="E128" s="5"/>
@@ -4757,7 +5272,7 @@
       <c r="A129" s="8"/>
       <c r="B129" s="8"/>
       <c r="C129" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D129" s="8"/>
       <c r="E129" s="5"/>
@@ -4767,7 +5282,7 @@
         <v>39</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C130" s="7">
         <v>5</v>
@@ -4779,7 +5294,7 @@
       <c r="A131" s="8"/>
       <c r="B131" s="8"/>
       <c r="C131" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D131" s="8"/>
       <c r="E131" s="5"/>
@@ -4788,7 +5303,7 @@
       <c r="A132" s="8"/>
       <c r="B132" s="8"/>
       <c r="C132" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D132" s="8"/>
       <c r="E132" s="5"/>
@@ -4797,10 +5312,10 @@
       <c r="A133" s="8"/>
       <c r="B133" s="8"/>
       <c r="C133" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E133" s="5"/>
     </row>
@@ -4808,10 +5323,10 @@
       <c r="A134" s="8"/>
       <c r="B134" s="8"/>
       <c r="C134" s="10" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E134" s="5"/>
     </row>
@@ -4819,10 +5334,10 @@
       <c r="A135" s="8"/>
       <c r="B135" s="8"/>
       <c r="C135" s="10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E135" s="5"/>
     </row>
@@ -4831,7 +5346,7 @@
         <v>40</v>
       </c>
       <c r="B136" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C136" s="7">
         <v>1</v>
@@ -4843,7 +5358,7 @@
       <c r="A137" s="8"/>
       <c r="B137" s="8"/>
       <c r="C137" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D137" s="8"/>
       <c r="E137" s="5"/>
@@ -4853,7 +5368,7 @@
         <v>41</v>
       </c>
       <c r="B138" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C138" s="7">
         <v>1</v>
@@ -4865,7 +5380,7 @@
       <c r="A139" s="8"/>
       <c r="B139" s="8"/>
       <c r="C139" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="5"/>
@@ -4875,7 +5390,7 @@
         <v>42</v>
       </c>
       <c r="B140" s="18" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C140" s="19">
         <v>1</v>
@@ -4887,7 +5402,7 @@
       <c r="A141" s="22"/>
       <c r="B141" s="23"/>
       <c r="C141" s="24" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D141" s="23"/>
       <c r="E141" s="25"/>
@@ -4897,7 +5412,7 @@
         <v>43</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C142" s="7">
         <v>2</v>
@@ -4909,10 +5424,10 @@
       <c r="A143" s="8"/>
       <c r="B143" s="8"/>
       <c r="C143" s="6" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E143" s="5"/>
     </row>
@@ -4920,7 +5435,7 @@
       <c r="A144" s="8"/>
       <c r="B144" s="8"/>
       <c r="C144" s="6" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="5"/>
@@ -4930,7 +5445,7 @@
         <v>44</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C145" s="7">
         <v>1</v>
@@ -4942,7 +5457,7 @@
       <c r="A146" s="8"/>
       <c r="B146" s="8"/>
       <c r="C146" s="6" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D146" s="8"/>
       <c r="E146" s="5"/>
@@ -4952,7 +5467,7 @@
         <v>45</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C147" s="7">
         <v>2</v>
@@ -4964,10 +5479,10 @@
       <c r="A148" s="8"/>
       <c r="B148" s="8"/>
       <c r="C148" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E148" s="5"/>
     </row>
@@ -4975,7 +5490,7 @@
       <c r="A149" s="8"/>
       <c r="B149" s="8"/>
       <c r="C149" s="6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D149" s="8"/>
       <c r="E149" s="5"/>
@@ -4985,7 +5500,7 @@
         <v>46</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C150" s="7">
         <v>1</v>
@@ -4997,10 +5512,10 @@
       <c r="A151" s="8"/>
       <c r="B151" s="8"/>
       <c r="C151" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E151" s="5"/>
     </row>
@@ -5011,4 +5526,89 @@
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC48D1F5-CB4E-EC46-91EA-0106B1CDEBBE}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added "animal" column to messel and rhynie, minor bug fixes
</commit_message>
<xml_diff>
--- a/data/rhynie/RhynieGuildStructure.xlsx
+++ b/data/rhynie/RhynieGuildStructure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tannerfrank/Dropbox/Work/Devonian terr ecosystems/EcolNetworks/RhynieWebRepo/data/rhynie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04812DE6-19A8-1B4A-BB07-6A41C4F78623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7A4759-46E8-1544-A674-DD159484C60F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="16580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guilds" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="265">
   <si>
     <t>guild_no</t>
   </si>
@@ -189,9 +189,6 @@
     <t>terrestrial nematodes</t>
   </si>
   <si>
-    <t>3,4,5,6,7,8,9,11,12,13,14,15,16,17,18,19,20,21,38</t>
-  </si>
-  <si>
     <t>terrestrial microbivores</t>
   </si>
   <si>
@@ -817,6 +814,9 @@
   </si>
   <si>
     <t>priority</t>
+  </si>
+  <si>
+    <t>animal</t>
   </si>
 </sst>
 </file>
@@ -2150,7 +2150,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1" customWidth="1"/>
@@ -2161,13 +2161,13 @@
     <col min="7" max="7" width="5.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="23" style="1" customWidth="1"/>
     <col min="9" max="9" width="26.6640625" style="1" customWidth="1"/>
-    <col min="10" max="11" width="10.83203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="12.6640625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="10" max="12" width="10.83203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2181,19 +2181,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>248</v>
-      </c>
       <c r="H1" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>260</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>4</v>
@@ -2202,10 +2202,13 @@
         <v>5</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>264</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -2239,11 +2242,14 @@
       <c r="K2" s="3">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -2260,7 +2266,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G3" s="3">
         <v>1</v>
@@ -2277,11 +2283,14 @@
       <c r="K3" s="3">
         <v>0</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -2298,7 +2307,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -2315,11 +2324,14 @@
       <c r="K4" s="3">
         <v>0</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="3">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -2336,7 +2348,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G5" s="3">
         <v>1</v>
@@ -2353,11 +2365,14 @@
       <c r="K5" s="3">
         <v>0</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="3">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -2374,7 +2389,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G6" s="3">
         <v>1</v>
@@ -2391,11 +2406,14 @@
       <c r="K6" s="3">
         <v>0</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="3">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -2412,7 +2430,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G7" s="3">
         <v>1</v>
@@ -2429,11 +2447,14 @@
       <c r="K7" s="3">
         <v>0</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="3">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -2450,7 +2471,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G8" s="3">
         <v>1</v>
@@ -2467,11 +2488,14 @@
       <c r="K8" s="3">
         <v>0</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="3">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -2486,7 +2510,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G9" s="3">
         <v>1</v>
@@ -2503,11 +2527,14 @@
       <c r="K9" s="3">
         <v>0</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="3">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -2522,7 +2549,7 @@
         <v>3</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G10" s="3">
         <v>1</v>
@@ -2539,11 +2566,14 @@
       <c r="K10" s="3">
         <v>0</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="3">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -2558,7 +2588,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G11" s="3">
         <v>1</v>
@@ -2575,9 +2605,12 @@
       <c r="K11" s="3">
         <v>0</v>
       </c>
-      <c r="L11" s="5"/>
-    </row>
-    <row r="12" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L11" s="3">
+        <v>0</v>
+      </c>
+      <c r="M11" s="5"/>
+    </row>
+    <row r="12" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -2594,7 +2627,7 @@
         <v>4</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G12" s="3">
         <v>1</v>
@@ -2612,10 +2645,13 @@
         <v>0</v>
       </c>
       <c r="L12" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -2630,7 +2666,7 @@
         <v>4</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G13" s="3">
         <v>1</v>
@@ -2647,9 +2683,12 @@
       <c r="K13" s="3">
         <v>0</v>
       </c>
-      <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L13" s="3">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -2664,7 +2703,7 @@
         <v>4</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G14" s="3">
         <v>1</v>
@@ -2681,9 +2720,12 @@
       <c r="K14" s="3">
         <v>0</v>
       </c>
-      <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L14" s="3">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -2698,7 +2740,7 @@
         <v>4</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G15" s="3">
         <v>1</v>
@@ -2715,9 +2757,12 @@
       <c r="K15" s="3">
         <v>0</v>
       </c>
-      <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L15" s="3">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -2732,7 +2777,7 @@
         <v>4</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G16" s="3">
         <v>1</v>
@@ -2749,9 +2794,12 @@
       <c r="K16" s="3">
         <v>0</v>
       </c>
-      <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" s="3">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2"/>
+    </row>
+    <row r="17" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -2768,7 +2816,7 @@
         <v>4</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G17" s="3">
         <v>1</v>
@@ -2785,11 +2833,14 @@
       <c r="K17" s="3">
         <v>0</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="3">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -2804,7 +2855,7 @@
         <v>4</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G18" s="3">
         <v>1</v>
@@ -2821,9 +2872,12 @@
       <c r="K18" s="3">
         <v>0</v>
       </c>
-      <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" s="3">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2"/>
+    </row>
+    <row r="19" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -2838,7 +2892,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G19" s="3">
         <v>1</v>
@@ -2855,9 +2909,12 @@
       <c r="K19" s="3">
         <v>0</v>
       </c>
-      <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" s="3">
+        <v>0</v>
+      </c>
+      <c r="M19" s="2"/>
+    </row>
+    <row r="20" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2872,7 +2929,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G20" s="3">
         <v>1</v>
@@ -2889,9 +2946,12 @@
       <c r="K20" s="3">
         <v>0</v>
       </c>
-      <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" s="3">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -2908,7 +2968,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G21" s="3">
         <v>1</v>
@@ -2925,11 +2985,14 @@
       <c r="K21" s="3">
         <v>0</v>
       </c>
-      <c r="L21" s="2" t="s">
+      <c r="L21" s="3">
+        <v>0</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2946,7 +3009,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G22" s="3">
         <v>1</v>
@@ -2963,11 +3026,14 @@
       <c r="K22" s="3">
         <v>0</v>
       </c>
-      <c r="L22" s="2" t="s">
+      <c r="L22" s="3">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -2991,7 +3057,7 @@
         <v>26</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="J23" s="3">
         <v>1</v>
@@ -2999,17 +3065,20 @@
       <c r="K23" s="3">
         <v>0</v>
       </c>
-      <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L23" s="3">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2"/>
+    </row>
+    <row r="24" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="D24" s="3">
         <v>1</v>
@@ -3018,7 +3087,7 @@
         <v>6</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G24" s="3">
         <v>1</v>
@@ -3027,27 +3096,30 @@
         <v>21</v>
       </c>
       <c r="I24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="J24" s="3">
+        <v>1</v>
+      </c>
+      <c r="K24" s="3">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J24" s="3">
-        <v>1</v>
-      </c>
-      <c r="K24" s="3">
-        <v>0</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D25" s="3">
         <v>2</v>
@@ -3056,36 +3128,39 @@
         <v>7</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G25" s="3">
         <v>2</v>
       </c>
       <c r="H25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="3">
+        <v>1</v>
+      </c>
+      <c r="K25" s="3">
+        <v>0</v>
+      </c>
+      <c r="L25" s="3">
+        <v>1</v>
+      </c>
+      <c r="M25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J25" s="3">
-        <v>1</v>
-      </c>
-      <c r="K25" s="3">
-        <v>0</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="D26" s="3">
         <v>2</v>
@@ -3094,7 +3169,7 @@
         <v>8</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G26" s="3">
         <v>2</v>
@@ -3103,27 +3178,30 @@
         <v>9</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J26" s="3">
+        <v>1</v>
+      </c>
+      <c r="K26" s="3">
+        <v>0</v>
+      </c>
+      <c r="L26" s="3">
+        <v>1</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="J26" s="3">
-        <v>1</v>
-      </c>
-      <c r="K26" s="3">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="D27" s="3">
         <v>3</v>
@@ -3132,7 +3210,7 @@
         <v>9</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G27" s="3">
         <v>3</v>
@@ -3141,7 +3219,7 @@
         <v>9</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J27" s="3">
         <v>1</v>
@@ -3149,19 +3227,22 @@
       <c r="K27" s="3">
         <v>0</v>
       </c>
-      <c r="L27" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L27" s="3">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="D28" s="3">
         <v>5</v>
@@ -3170,7 +3251,7 @@
         <v>10</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G28" s="3">
         <v>5</v>
@@ -3179,24 +3260,27 @@
         <v>9</v>
       </c>
       <c r="I28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J28" s="3">
+        <v>1</v>
+      </c>
+      <c r="K28" s="3">
+        <v>0</v>
+      </c>
+      <c r="L28" s="3">
+        <v>1</v>
+      </c>
+      <c r="M28" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J28" s="3">
-        <v>1</v>
-      </c>
-      <c r="K28" s="3">
-        <v>0</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>7</v>
@@ -3208,7 +3292,7 @@
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G29" s="3">
         <v>1</v>
@@ -3225,16 +3309,19 @@
       <c r="K29" s="3">
         <v>1</v>
       </c>
-      <c r="L29" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L29" s="3">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="3">
@@ -3244,33 +3331,36 @@
         <v>12</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G30" s="3">
         <v>1</v>
       </c>
       <c r="H30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
+        <v>1</v>
+      </c>
+      <c r="L30" s="3">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="J30" s="3">
-        <v>0</v>
-      </c>
-      <c r="K30" s="3">
-        <v>1</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="3">
@@ -3280,7 +3370,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G31" s="3">
         <v>1</v>
@@ -3297,14 +3387,17 @@
       <c r="K31" s="3">
         <v>1</v>
       </c>
-      <c r="L31" s="5"/>
-    </row>
-    <row r="32" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L31" s="3">
+        <v>0</v>
+      </c>
+      <c r="M31" s="5"/>
+    </row>
+    <row r="32" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="3">
@@ -3314,31 +3407,34 @@
         <v>12</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G32" s="3">
         <v>1</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I32" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="J32" s="3">
         <v>0</v>
       </c>
       <c r="K32" s="3">
         <v>1</v>
       </c>
-      <c r="L32" s="5"/>
-    </row>
-    <row r="33" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L32" s="3">
+        <v>0</v>
+      </c>
+      <c r="M32" s="5"/>
+    </row>
+    <row r="33" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="3">
@@ -3348,7 +3444,7 @@
         <v>13</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G33" s="3">
         <v>1</v>
@@ -3365,17 +3461,20 @@
       <c r="K33" s="3">
         <v>1</v>
       </c>
-      <c r="L33" s="5"/>
-    </row>
-    <row r="34" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L33" s="3">
+        <v>0</v>
+      </c>
+      <c r="M33" s="5"/>
+    </row>
+    <row r="34" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="D34" s="3">
         <v>5</v>
@@ -3384,7 +3483,7 @@
         <v>13</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G34" s="3">
         <v>1</v>
@@ -3401,17 +3500,20 @@
       <c r="K34" s="3">
         <v>1</v>
       </c>
-      <c r="L34" s="5"/>
-    </row>
-    <row r="35" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L34" s="3">
+        <v>0</v>
+      </c>
+      <c r="M34" s="5"/>
+    </row>
+    <row r="35" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
@@ -3420,7 +3522,7 @@
         <v>13</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G35" s="3">
         <v>1</v>
@@ -3437,17 +3539,20 @@
       <c r="K35" s="3">
         <v>1</v>
       </c>
-      <c r="L35" s="5"/>
-    </row>
-    <row r="36" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L35" s="3">
+        <v>0</v>
+      </c>
+      <c r="M35" s="5"/>
+    </row>
+    <row r="36" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D36" s="3">
         <v>5</v>
@@ -3456,7 +3561,7 @@
         <v>13</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G36" s="3">
         <v>1</v>
@@ -3473,17 +3578,20 @@
       <c r="K36" s="3">
         <v>1</v>
       </c>
-      <c r="L36" s="5"/>
-    </row>
-    <row r="37" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L36" s="3">
+        <v>0</v>
+      </c>
+      <c r="M36" s="5"/>
+    </row>
+    <row r="37" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37" s="3">
         <v>4</v>
@@ -3492,7 +3600,7 @@
         <v>13</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G37" s="3">
         <v>1</v>
@@ -3509,17 +3617,20 @@
       <c r="K37" s="3">
         <v>1</v>
       </c>
-      <c r="L37" s="5"/>
-    </row>
-    <row r="38" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L37" s="3">
+        <v>0</v>
+      </c>
+      <c r="M37" s="5"/>
+    </row>
+    <row r="38" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="D38" s="3">
         <v>1</v>
@@ -3528,7 +3639,7 @@
         <v>14</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G38" s="3">
         <v>1</v>
@@ -3545,17 +3656,20 @@
       <c r="K38" s="3">
         <v>1</v>
       </c>
-      <c r="L38" s="5"/>
-    </row>
-    <row r="39" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L38" s="3">
+        <v>0</v>
+      </c>
+      <c r="M38" s="5"/>
+    </row>
+    <row r="39" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="D39" s="3">
         <v>3</v>
@@ -3564,7 +3678,7 @@
         <v>13</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G39" s="3">
         <v>1</v>
@@ -3581,14 +3695,17 @@
       <c r="K39" s="3">
         <v>1</v>
       </c>
-      <c r="L39" s="5"/>
-    </row>
-    <row r="40" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L39" s="3">
+        <v>0</v>
+      </c>
+      <c r="M39" s="5"/>
+    </row>
+    <row r="40" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>49</v>
@@ -3600,7 +3717,7 @@
         <v>15</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G40" s="3">
         <v>1</v>
@@ -3618,15 +3735,18 @@
         <v>1</v>
       </c>
       <c r="L40" s="3">
+        <v>0</v>
+      </c>
+      <c r="M40" s="3">
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>49</v>
@@ -3638,33 +3758,36 @@
         <v>15</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G41" s="3">
         <v>1</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3">
+        <v>1</v>
+      </c>
+      <c r="L41" s="3">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="J41" s="3">
-        <v>0</v>
-      </c>
-      <c r="K41" s="3">
-        <v>1</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>49</v>
@@ -3676,7 +3799,7 @@
         <v>15</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G42" s="3">
         <v>1</v>
@@ -3685,27 +3808,30 @@
         <v>9</v>
       </c>
       <c r="I42" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J42" s="3">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3">
+        <v>1</v>
+      </c>
+      <c r="L42" s="3">
+        <v>0</v>
+      </c>
+      <c r="M42" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="J42" s="3">
-        <v>0</v>
-      </c>
-      <c r="K42" s="3">
-        <v>1</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="D43" s="3">
         <v>1</v>
@@ -3714,7 +3840,7 @@
         <v>16</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G43" s="3">
         <v>1</v>
@@ -3723,27 +3849,30 @@
         <v>9</v>
       </c>
       <c r="I43" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J43" s="3">
+        <v>0</v>
+      </c>
+      <c r="K43" s="3">
+        <v>1</v>
+      </c>
+      <c r="L43" s="3">
+        <v>1</v>
+      </c>
+      <c r="M43" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="J43" s="3">
-        <v>0</v>
-      </c>
-      <c r="K43" s="3">
-        <v>1</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="D44" s="3">
         <v>2</v>
@@ -3752,7 +3881,7 @@
         <v>17</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G44" s="3">
         <v>2</v>
@@ -3761,27 +3890,30 @@
         <v>9</v>
       </c>
       <c r="I44" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3">
+        <v>1</v>
+      </c>
+      <c r="L44" s="3">
+        <v>1</v>
+      </c>
+      <c r="M44" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="J44" s="3">
-        <v>0</v>
-      </c>
-      <c r="K44" s="3">
-        <v>1</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D45" s="3">
         <v>1</v>
@@ -3790,36 +3922,39 @@
         <v>18</v>
       </c>
       <c r="F45" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G45" s="3">
+        <v>1</v>
+      </c>
+      <c r="H45" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="G45" s="3">
-        <v>1</v>
-      </c>
-      <c r="H45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="J45" s="3">
+        <v>0</v>
+      </c>
+      <c r="K45" s="3">
+        <v>1</v>
+      </c>
+      <c r="L45" s="3">
+        <v>1</v>
+      </c>
+      <c r="M45" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="J45" s="3">
-        <v>0</v>
-      </c>
-      <c r="K45" s="3">
-        <v>1</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="D46" s="3">
         <v>2</v>
@@ -3828,7 +3963,7 @@
         <v>19</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G46" s="3">
         <v>2</v>
@@ -3837,27 +3972,30 @@
         <v>9</v>
       </c>
       <c r="I46" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0</v>
+      </c>
+      <c r="K46" s="3">
+        <v>1</v>
+      </c>
+      <c r="L46" s="3">
+        <v>1</v>
+      </c>
+      <c r="M46" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="J46" s="3">
-        <v>0</v>
-      </c>
-      <c r="K46" s="3">
-        <v>1</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="D47" s="3">
         <v>1</v>
@@ -3866,7 +4004,7 @@
         <v>20</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G47" s="3">
         <v>1</v>
@@ -3875,16 +4013,19 @@
         <v>9</v>
       </c>
       <c r="I47" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="3">
+        <v>1</v>
+      </c>
+      <c r="L47" s="3">
+        <v>1</v>
+      </c>
+      <c r="M47" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="J47" s="3">
-        <v>0</v>
-      </c>
-      <c r="K47" s="3">
-        <v>1</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3910,16 +4051,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="E1" s="5"/>
     </row>
@@ -3940,7 +4081,7 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="5"/>
@@ -3962,7 +4103,7 @@
       <c r="A5" s="9"/>
       <c r="B5" s="4"/>
       <c r="C5" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="5"/>
@@ -3984,7 +4125,7 @@
       <c r="A7" s="9"/>
       <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="5"/>
@@ -4006,7 +4147,7 @@
       <c r="A9" s="9"/>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="5"/>
@@ -4028,7 +4169,7 @@
       <c r="A11" s="9"/>
       <c r="B11" s="4"/>
       <c r="C11" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="5"/>
@@ -4050,7 +4191,7 @@
       <c r="A13" s="9"/>
       <c r="B13" s="6"/>
       <c r="C13" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="5"/>
@@ -4072,7 +4213,7 @@
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="5"/>
@@ -4081,7 +4222,7 @@
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="5"/>
@@ -4101,7 +4242,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="5"/>
@@ -4110,7 +4251,7 @@
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="5"/>
@@ -4132,7 +4273,7 @@
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="5"/>
@@ -4154,10 +4295,10 @@
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>138</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>139</v>
       </c>
       <c r="E23" s="5"/>
     </row>
@@ -4178,7 +4319,7 @@
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="5"/>
@@ -4187,10 +4328,10 @@
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>142</v>
       </c>
       <c r="E26" s="5"/>
     </row>
@@ -4198,10 +4339,10 @@
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E27" s="5"/>
     </row>
@@ -4209,10 +4350,10 @@
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E28" s="5"/>
     </row>
@@ -4220,10 +4361,10 @@
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E29" s="5"/>
     </row>
@@ -4231,10 +4372,10 @@
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E30" s="5"/>
     </row>
@@ -4242,7 +4383,7 @@
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="5"/>
@@ -4251,7 +4392,7 @@
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="5"/>
@@ -4260,7 +4401,7 @@
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="5"/>
@@ -4269,7 +4410,7 @@
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
@@ -4278,7 +4419,7 @@
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="5"/>
@@ -4287,7 +4428,7 @@
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="5"/>
@@ -4296,10 +4437,10 @@
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E37" s="5"/>
     </row>
@@ -4307,10 +4448,10 @@
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E38" s="5"/>
     </row>
@@ -4331,7 +4472,7 @@
       <c r="A40" s="9"/>
       <c r="B40" s="6"/>
       <c r="C40" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="5"/>
@@ -4340,7 +4481,7 @@
       <c r="A41" s="9"/>
       <c r="B41" s="6"/>
       <c r="C41" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="5"/>
@@ -4349,7 +4490,7 @@
       <c r="A42" s="9"/>
       <c r="B42" s="6"/>
       <c r="C42" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="5"/>
@@ -4371,7 +4512,7 @@
       <c r="A44" s="9"/>
       <c r="B44" s="6"/>
       <c r="C44" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="5"/>
@@ -4380,7 +4521,7 @@
       <c r="A45" s="9"/>
       <c r="B45" s="6"/>
       <c r="C45" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="5"/>
@@ -4402,7 +4543,7 @@
       <c r="A47" s="9"/>
       <c r="B47" s="6"/>
       <c r="C47" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="5"/>
@@ -4411,7 +4552,7 @@
       <c r="A48" s="9"/>
       <c r="B48" s="6"/>
       <c r="C48" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="5"/>
@@ -4420,7 +4561,7 @@
       <c r="A49" s="9"/>
       <c r="B49" s="6"/>
       <c r="C49" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="5"/>
@@ -4442,7 +4583,7 @@
       <c r="A51" s="9"/>
       <c r="B51" s="6"/>
       <c r="C51" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="5"/>
@@ -4451,7 +4592,7 @@
       <c r="A52" s="9"/>
       <c r="B52" s="6"/>
       <c r="C52" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="5"/>
@@ -4460,7 +4601,7 @@
       <c r="A53" s="9"/>
       <c r="B53" s="6"/>
       <c r="C53" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="5"/>
@@ -4482,10 +4623,10 @@
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="D55" s="10" t="s">
         <v>165</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>166</v>
       </c>
       <c r="E55" s="5"/>
     </row>
@@ -4506,7 +4647,7 @@
       <c r="A57" s="9"/>
       <c r="B57" s="6"/>
       <c r="C57" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D57" s="8"/>
       <c r="E57" s="5"/>
@@ -4528,10 +4669,10 @@
       <c r="A59" s="9"/>
       <c r="B59" s="6"/>
       <c r="C59" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E59" s="5"/>
     </row>
@@ -4539,7 +4680,7 @@
       <c r="A60" s="9"/>
       <c r="B60" s="6"/>
       <c r="C60" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D60" s="8"/>
       <c r="E60" s="5"/>
@@ -4548,7 +4689,7 @@
       <c r="A61" s="9"/>
       <c r="B61" s="6"/>
       <c r="C61" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D61" s="8"/>
       <c r="E61" s="5"/>
@@ -4570,10 +4711,10 @@
       <c r="A63" s="9"/>
       <c r="B63" s="6"/>
       <c r="C63" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E63" s="5"/>
     </row>
@@ -4582,7 +4723,7 @@
         <v>20</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C64" s="7">
         <v>2</v>
@@ -4594,7 +4735,7 @@
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
@@ -4603,10 +4744,10 @@
       <c r="A66" s="8"/>
       <c r="B66" s="8"/>
       <c r="C66" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E66" s="5"/>
     </row>
@@ -4627,10 +4768,10 @@
       <c r="A68" s="8"/>
       <c r="B68" s="8"/>
       <c r="C68" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D68" s="10" t="s">
         <v>175</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>176</v>
       </c>
       <c r="E68" s="5"/>
     </row>
@@ -4638,10 +4779,10 @@
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E69" s="5"/>
     </row>
@@ -4649,10 +4790,10 @@
       <c r="A70" s="8"/>
       <c r="B70" s="8"/>
       <c r="C70" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E70" s="5"/>
     </row>
@@ -4660,10 +4801,10 @@
       <c r="A71" s="8"/>
       <c r="B71" s="8"/>
       <c r="C71" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E71" s="5"/>
     </row>
@@ -4671,10 +4812,10 @@
       <c r="A72" s="8"/>
       <c r="B72" s="8"/>
       <c r="C72" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>181</v>
       </c>
       <c r="E72" s="5"/>
     </row>
@@ -4682,10 +4823,10 @@
       <c r="A73" s="8"/>
       <c r="B73" s="8"/>
       <c r="C73" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D73" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>183</v>
       </c>
       <c r="E73" s="5"/>
     </row>
@@ -4693,10 +4834,10 @@
       <c r="A74" s="8"/>
       <c r="B74" s="8"/>
       <c r="C74" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D74" s="6" t="s">
         <v>184</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>185</v>
       </c>
       <c r="E74" s="5"/>
     </row>
@@ -4717,7 +4858,7 @@
       <c r="A76" s="9"/>
       <c r="B76" s="6"/>
       <c r="C76" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D76" s="8"/>
       <c r="E76" s="5"/>
@@ -4727,7 +4868,7 @@
         <v>23</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C77" s="7">
         <v>1</v>
@@ -4739,7 +4880,7 @@
       <c r="A78" s="8"/>
       <c r="B78" s="8"/>
       <c r="C78" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D78" s="8"/>
       <c r="E78" s="5"/>
@@ -4749,7 +4890,7 @@
         <v>24</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C79" s="7">
         <v>2</v>
@@ -4761,10 +4902,10 @@
       <c r="A80" s="8"/>
       <c r="B80" s="8"/>
       <c r="C80" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E80" s="5"/>
     </row>
@@ -4772,7 +4913,7 @@
       <c r="A81" s="8"/>
       <c r="B81" s="8"/>
       <c r="C81" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D81" s="8"/>
       <c r="E81" s="5"/>
@@ -4782,7 +4923,7 @@
         <v>25</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C82" s="7">
         <v>2</v>
@@ -4794,10 +4935,10 @@
       <c r="A83" s="8"/>
       <c r="B83" s="8"/>
       <c r="C83" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E83" s="5"/>
     </row>
@@ -4805,10 +4946,10 @@
       <c r="A84" s="8"/>
       <c r="B84" s="8"/>
       <c r="C84" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E84" s="5"/>
     </row>
@@ -4817,7 +4958,7 @@
         <v>26</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C85" s="7">
         <v>3</v>
@@ -4829,7 +4970,7 @@
       <c r="A86" s="8"/>
       <c r="B86" s="8"/>
       <c r="C86" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D86" s="8"/>
       <c r="E86" s="5"/>
@@ -4838,7 +4979,7 @@
       <c r="A87" s="8"/>
       <c r="B87" s="8"/>
       <c r="C87" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D87" s="8"/>
       <c r="E87" s="5"/>
@@ -4847,7 +4988,7 @@
       <c r="A88" s="8"/>
       <c r="B88" s="8"/>
       <c r="C88" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D88" s="8"/>
       <c r="E88" s="5"/>
@@ -4857,7 +4998,7 @@
         <v>27</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C89" s="7">
         <v>5</v>
@@ -4869,7 +5010,7 @@
       <c r="A90" s="8"/>
       <c r="B90" s="8"/>
       <c r="C90" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D90" s="8"/>
       <c r="E90" s="5"/>
@@ -4878,7 +5019,7 @@
       <c r="A91" s="8"/>
       <c r="B91" s="8"/>
       <c r="C91" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D91" s="8"/>
       <c r="E91" s="5"/>
@@ -4887,7 +5028,7 @@
       <c r="A92" s="8"/>
       <c r="B92" s="8"/>
       <c r="C92" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D92" s="8"/>
       <c r="E92" s="5"/>
@@ -4896,7 +5037,7 @@
       <c r="A93" s="8"/>
       <c r="B93" s="8"/>
       <c r="C93" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D93" s="8"/>
       <c r="E93" s="5"/>
@@ -4905,7 +5046,7 @@
       <c r="A94" s="8"/>
       <c r="B94" s="8"/>
       <c r="C94" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D94" s="8"/>
       <c r="E94" s="5"/>
@@ -4915,7 +5056,7 @@
         <v>28</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C95" s="7">
         <v>1</v>
@@ -4927,7 +5068,7 @@
       <c r="A96" s="8"/>
       <c r="B96" s="8"/>
       <c r="C96" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D96" s="8"/>
       <c r="E96" s="5"/>
@@ -4937,7 +5078,7 @@
         <v>29</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C97" s="7">
         <v>1</v>
@@ -4949,7 +5090,7 @@
       <c r="A98" s="8"/>
       <c r="B98" s="8"/>
       <c r="C98" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D98" s="8"/>
       <c r="E98" s="5"/>
@@ -4959,7 +5100,7 @@
         <v>30</v>
       </c>
       <c r="B99" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C99" s="7">
         <v>1</v>
@@ -4971,7 +5112,7 @@
       <c r="A100" s="8"/>
       <c r="B100" s="8"/>
       <c r="C100" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D100" s="8"/>
       <c r="E100" s="5"/>
@@ -4981,7 +5122,7 @@
         <v>31</v>
       </c>
       <c r="B101" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C101" s="3">
         <v>1</v>
@@ -4993,7 +5134,7 @@
       <c r="A102" s="8"/>
       <c r="B102" s="8"/>
       <c r="C102" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D102" s="8"/>
       <c r="E102" s="5"/>
@@ -5003,7 +5144,7 @@
         <v>32</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C103" s="3">
         <v>1</v>
@@ -5015,7 +5156,7 @@
       <c r="A104" s="9"/>
       <c r="B104" s="6"/>
       <c r="C104" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D104" s="8"/>
       <c r="E104" s="5"/>
@@ -5025,7 +5166,7 @@
         <v>33</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C105" s="7">
         <v>5</v>
@@ -5037,7 +5178,7 @@
       <c r="A106" s="8"/>
       <c r="B106" s="8"/>
       <c r="C106" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D106" s="8"/>
       <c r="E106" s="5"/>
@@ -5046,7 +5187,7 @@
       <c r="A107" s="8"/>
       <c r="B107" s="8"/>
       <c r="C107" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D107" s="8"/>
       <c r="E107" s="5"/>
@@ -5055,7 +5196,7 @@
       <c r="A108" s="8"/>
       <c r="B108" s="8"/>
       <c r="C108" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="5"/>
@@ -5064,7 +5205,7 @@
       <c r="A109" s="8"/>
       <c r="B109" s="8"/>
       <c r="C109" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D109" s="8"/>
       <c r="E109" s="5"/>
@@ -5073,7 +5214,7 @@
       <c r="A110" s="8"/>
       <c r="B110" s="8"/>
       <c r="C110" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D110" s="8"/>
       <c r="E110" s="5"/>
@@ -5083,7 +5224,7 @@
         <v>34</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C111" s="7">
         <v>1</v>
@@ -5095,7 +5236,7 @@
       <c r="A112" s="8"/>
       <c r="B112" s="8"/>
       <c r="C112" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D112" s="8"/>
       <c r="E112" s="5"/>
@@ -5105,7 +5246,7 @@
         <v>35</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C113" s="7">
         <v>5</v>
@@ -5117,10 +5258,10 @@
       <c r="A114" s="8"/>
       <c r="B114" s="8"/>
       <c r="C114" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D114" s="6" t="s">
         <v>214</v>
-      </c>
-      <c r="D114" s="6" t="s">
-        <v>215</v>
       </c>
       <c r="E114" s="5"/>
     </row>
@@ -5128,10 +5269,10 @@
       <c r="A115" s="8"/>
       <c r="B115" s="8"/>
       <c r="C115" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E115" s="5"/>
     </row>
@@ -5139,7 +5280,7 @@
       <c r="A116" s="8"/>
       <c r="B116" s="8"/>
       <c r="C116" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D116" s="8"/>
       <c r="E116" s="5"/>
@@ -5148,10 +5289,10 @@
       <c r="A117" s="8"/>
       <c r="B117" s="8"/>
       <c r="C117" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E117" s="5"/>
     </row>
@@ -5159,10 +5300,10 @@
       <c r="A118" s="8"/>
       <c r="B118" s="8"/>
       <c r="C118" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="D118" s="6" t="s">
         <v>219</v>
-      </c>
-      <c r="D118" s="6" t="s">
-        <v>220</v>
       </c>
       <c r="E118" s="5"/>
     </row>
@@ -5171,7 +5312,7 @@
         <v>36</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C119" s="7">
         <v>4</v>
@@ -5183,7 +5324,7 @@
       <c r="A120" s="8"/>
       <c r="B120" s="8"/>
       <c r="C120" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D120" s="8"/>
       <c r="E120" s="5"/>
@@ -5192,7 +5333,7 @@
       <c r="A121" s="8"/>
       <c r="B121" s="8"/>
       <c r="C121" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D121" s="8"/>
       <c r="E121" s="5"/>
@@ -5201,7 +5342,7 @@
       <c r="A122" s="8"/>
       <c r="B122" s="8"/>
       <c r="C122" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D122" s="8"/>
       <c r="E122" s="5"/>
@@ -5210,7 +5351,7 @@
       <c r="A123" s="8"/>
       <c r="B123" s="8"/>
       <c r="C123" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D123" s="8"/>
       <c r="E123" s="5"/>
@@ -5220,7 +5361,7 @@
         <v>37</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C124" s="7">
         <v>1</v>
@@ -5232,7 +5373,7 @@
       <c r="A125" s="8"/>
       <c r="B125" s="8"/>
       <c r="C125" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D125" s="8"/>
       <c r="E125" s="5"/>
@@ -5242,7 +5383,7 @@
         <v>38</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C126" s="16">
         <v>3</v>
@@ -5254,7 +5395,7 @@
       <c r="A127" s="8"/>
       <c r="B127" s="8"/>
       <c r="C127" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D127" s="8"/>
       <c r="E127" s="5"/>
@@ -5263,7 +5404,7 @@
       <c r="A128" s="8"/>
       <c r="B128" s="8"/>
       <c r="C128" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D128" s="8"/>
       <c r="E128" s="5"/>
@@ -5272,7 +5413,7 @@
       <c r="A129" s="8"/>
       <c r="B129" s="8"/>
       <c r="C129" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D129" s="8"/>
       <c r="E129" s="5"/>
@@ -5282,7 +5423,7 @@
         <v>39</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C130" s="7">
         <v>5</v>
@@ -5294,7 +5435,7 @@
       <c r="A131" s="8"/>
       <c r="B131" s="8"/>
       <c r="C131" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D131" s="8"/>
       <c r="E131" s="5"/>
@@ -5303,7 +5444,7 @@
       <c r="A132" s="8"/>
       <c r="B132" s="8"/>
       <c r="C132" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D132" s="8"/>
       <c r="E132" s="5"/>
@@ -5312,10 +5453,10 @@
       <c r="A133" s="8"/>
       <c r="B133" s="8"/>
       <c r="C133" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E133" s="5"/>
     </row>
@@ -5323,10 +5464,10 @@
       <c r="A134" s="8"/>
       <c r="B134" s="8"/>
       <c r="C134" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E134" s="5"/>
     </row>
@@ -5334,10 +5475,10 @@
       <c r="A135" s="8"/>
       <c r="B135" s="8"/>
       <c r="C135" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E135" s="5"/>
     </row>
@@ -5346,7 +5487,7 @@
         <v>40</v>
       </c>
       <c r="B136" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C136" s="7">
         <v>1</v>
@@ -5358,7 +5499,7 @@
       <c r="A137" s="8"/>
       <c r="B137" s="8"/>
       <c r="C137" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D137" s="8"/>
       <c r="E137" s="5"/>
@@ -5368,7 +5509,7 @@
         <v>41</v>
       </c>
       <c r="B138" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C138" s="7">
         <v>1</v>
@@ -5380,7 +5521,7 @@
       <c r="A139" s="8"/>
       <c r="B139" s="8"/>
       <c r="C139" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="5"/>
@@ -5390,7 +5531,7 @@
         <v>42</v>
       </c>
       <c r="B140" s="18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C140" s="19">
         <v>1</v>
@@ -5402,7 +5543,7 @@
       <c r="A141" s="22"/>
       <c r="B141" s="23"/>
       <c r="C141" s="24" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D141" s="23"/>
       <c r="E141" s="25"/>
@@ -5412,7 +5553,7 @@
         <v>43</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C142" s="7">
         <v>2</v>
@@ -5424,10 +5565,10 @@
       <c r="A143" s="8"/>
       <c r="B143" s="8"/>
       <c r="C143" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E143" s="5"/>
     </row>
@@ -5435,7 +5576,7 @@
       <c r="A144" s="8"/>
       <c r="B144" s="8"/>
       <c r="C144" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="5"/>
@@ -5445,7 +5586,7 @@
         <v>44</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C145" s="7">
         <v>1</v>
@@ -5457,7 +5598,7 @@
       <c r="A146" s="8"/>
       <c r="B146" s="8"/>
       <c r="C146" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D146" s="8"/>
       <c r="E146" s="5"/>
@@ -5467,7 +5608,7 @@
         <v>45</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C147" s="7">
         <v>2</v>
@@ -5479,10 +5620,10 @@
       <c r="A148" s="8"/>
       <c r="B148" s="8"/>
       <c r="C148" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E148" s="5"/>
     </row>
@@ -5490,7 +5631,7 @@
       <c r="A149" s="8"/>
       <c r="B149" s="8"/>
       <c r="C149" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D149" s="8"/>
       <c r="E149" s="5"/>
@@ -5500,7 +5641,7 @@
         <v>46</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C150" s="7">
         <v>1</v>
@@ -5512,10 +5653,10 @@
       <c r="A151" s="8"/>
       <c r="B151" s="8"/>
       <c r="C151" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E151" s="5"/>
     </row>
@@ -5540,16 +5681,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" t="s">
         <v>256</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D1" t="s">
         <v>257</v>
-      </c>
-      <c r="C1" t="s">
-        <v>264</v>
-      </c>
-      <c r="D1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -5563,7 +5704,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -5577,7 +5718,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -5591,7 +5732,7 @@
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -5605,7 +5746,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>